<commit_message>
Checkpoint: before performance optimization
</commit_message>
<xml_diff>
--- a/Product List.xlsx
+++ b/Product List.xlsx
@@ -883,7 +883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3155"/>
+  <dimension ref="A1:C3169"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="55.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -50431,6 +50431,244 @@
       <c r="C3155" t="inlineStr">
         <is>
           <t>pumpss</t>
+        </is>
+      </c>
+    </row>
+    <row r="3156">
+      <c r="A3156" t="inlineStr">
+        <is>
+          <t>471 TC-4BX</t>
+        </is>
+      </c>
+      <c r="B3156" t="inlineStr">
+        <is>
+          <t>PARKER</t>
+        </is>
+      </c>
+      <c r="C3156" t="inlineStr">
+        <is>
+          <t>hydraulic hose 1/2"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3157">
+      <c r="A3157" t="inlineStr">
+        <is>
+          <t>471 TC-8BX</t>
+        </is>
+      </c>
+      <c r="B3157" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C3157" t="inlineStr">
+        <is>
+          <t>HYDRAULIC HOSE 1/2"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3158">
+      <c r="A3158" t="inlineStr">
+        <is>
+          <t>471 TC 12BX</t>
+        </is>
+      </c>
+      <c r="B3158" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C3158" t="inlineStr">
+        <is>
+          <t>HYDRAULIC HOSE 3/4 "</t>
+        </is>
+      </c>
+    </row>
+    <row r="3159">
+      <c r="A3159" t="inlineStr">
+        <is>
+          <t>471 TC- 16BX</t>
+        </is>
+      </c>
+      <c r="B3159" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C3159" t="inlineStr">
+        <is>
+          <t>HYDRAULIC HOSE 1"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3160">
+      <c r="A3160" t="inlineStr">
+        <is>
+          <t>471 TC- 20BX</t>
+        </is>
+      </c>
+      <c r="B3160" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C3160" t="inlineStr">
+        <is>
+          <t>HYDRAULIC HOSE 1 1/4"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3161">
+      <c r="A3161" t="inlineStr">
+        <is>
+          <t>10643-4-4</t>
+        </is>
+      </c>
+      <c r="B3161" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C3161" t="inlineStr">
+        <is>
+          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3162">
+      <c r="A3162" t="inlineStr">
+        <is>
+          <t>10643-8-8</t>
+        </is>
+      </c>
+      <c r="B3162" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C3162" t="inlineStr">
+        <is>
+          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3163">
+      <c r="A3163" t="inlineStr">
+        <is>
+          <t>10643-12-12</t>
+        </is>
+      </c>
+      <c r="B3163" t="inlineStr">
+        <is>
+          <t>PARKER</t>
+        </is>
+      </c>
+      <c r="C3163" t="inlineStr">
+        <is>
+          <t>JIC 37`, FEMALE, SWIVEL, 90` ELBOW SIZE 3/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3164">
+      <c r="A3164" t="inlineStr">
+        <is>
+          <t>10643-16-16</t>
+        </is>
+      </c>
+      <c r="B3164" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C3164" t="inlineStr">
+        <is>
+          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3165">
+      <c r="A3165" t="inlineStr">
+        <is>
+          <t>10643-20-20</t>
+        </is>
+      </c>
+      <c r="B3165" t="inlineStr">
+        <is>
+          <t>GENERAL</t>
+        </is>
+      </c>
+      <c r="C3165" t="inlineStr">
+        <is>
+          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1 1/4"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3166">
+      <c r="A3166" t="inlineStr">
+        <is>
+          <t>472 TC-20</t>
+        </is>
+      </c>
+      <c r="B3166" t="inlineStr">
+        <is>
+          <t>PARKER</t>
+        </is>
+      </c>
+      <c r="C3166" t="inlineStr">
+        <is>
+          <t>HYDRAULIC HOSE 1 1/4 "</t>
+        </is>
+      </c>
+    </row>
+    <row r="3167">
+      <c r="A3167" t="inlineStr">
+        <is>
+          <t>13943-8-8</t>
+        </is>
+      </c>
+      <c r="B3167" t="inlineStr">
+        <is>
+          <t>PARKER</t>
+        </is>
+      </c>
+      <c r="C3167" t="inlineStr">
+        <is>
+          <t>JIC 37`, FEMALE, SWIVEL, 90` ELBOW SIZE 1/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3168">
+      <c r="A3168" t="inlineStr">
+        <is>
+          <t>13943-12-12</t>
+        </is>
+      </c>
+      <c r="B3168" t="inlineStr">
+        <is>
+          <t>PARKER</t>
+        </is>
+      </c>
+      <c r="C3168" t="inlineStr">
+        <is>
+          <t>JIC 37`, FEMALE, SWIVEL, 90` ELBOW SIZE 3/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3169">
+      <c r="A3169" t="inlineStr">
+        <is>
+          <t>13943-16-16</t>
+        </is>
+      </c>
+      <c r="B3169" t="inlineStr">
+        <is>
+          <t>PARKER</t>
+        </is>
+      </c>
+      <c r="C3169" t="inlineStr">
+        <is>
+          <t>JIC 37`, FEMALE, SWIVEL, 90` ELBOW SIZE 1 1/4"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update quotation workflow: optional item description, date auto-fill, save-to-catalog modal, expanded HSN box, and 2-page PDF layout
</commit_message>
<xml_diff>
--- a/Product List.xlsx
+++ b/Product List.xlsx
@@ -883,7 +883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3169"/>
+  <dimension ref="A1:C3168"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col width="55.5703125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -50403,58 +50403,58 @@
     <row r="3154">
       <c r="A3154" t="inlineStr">
         <is>
-          <t>99999999999</t>
+          <t>88888888</t>
         </is>
       </c>
       <c r="B3154" t="inlineStr">
         <is>
-          <t>DANFOSS</t>
+          <t>GENERAL</t>
         </is>
       </c>
       <c r="C3154" t="inlineStr">
         <is>
-          <t>PUMPSt</t>
+          <t>pumpss</t>
         </is>
       </c>
     </row>
     <row r="3155">
       <c r="A3155" t="inlineStr">
         <is>
-          <t>88888888</t>
+          <t>471 TC-4BX</t>
         </is>
       </c>
       <c r="B3155" t="inlineStr">
         <is>
-          <t>GENERAL</t>
+          <t>PARKER</t>
         </is>
       </c>
       <c r="C3155" t="inlineStr">
         <is>
-          <t>pumpss</t>
+          <t>hydraulic hose 1/2"</t>
         </is>
       </c>
     </row>
     <row r="3156">
       <c r="A3156" t="inlineStr">
         <is>
-          <t>471 TC-4BX</t>
+          <t>471 TC-8BX</t>
         </is>
       </c>
       <c r="B3156" t="inlineStr">
         <is>
-          <t>PARKER</t>
+          <t>GENERAL</t>
         </is>
       </c>
       <c r="C3156" t="inlineStr">
         <is>
-          <t>hydraulic hose 1/2"</t>
+          <t>HYDRAULIC HOSE 1/2"</t>
         </is>
       </c>
     </row>
     <row r="3157">
       <c r="A3157" t="inlineStr">
         <is>
-          <t>471 TC-8BX</t>
+          <t>471 TC 12BX</t>
         </is>
       </c>
       <c r="B3157" t="inlineStr">
@@ -50464,14 +50464,14 @@
       </c>
       <c r="C3157" t="inlineStr">
         <is>
-          <t>HYDRAULIC HOSE 1/2"</t>
+          <t>HYDRAULIC HOSE 3/4 "</t>
         </is>
       </c>
     </row>
     <row r="3158">
       <c r="A3158" t="inlineStr">
         <is>
-          <t>471 TC 12BX</t>
+          <t>471 TC- 16BX</t>
         </is>
       </c>
       <c r="B3158" t="inlineStr">
@@ -50481,14 +50481,14 @@
       </c>
       <c r="C3158" t="inlineStr">
         <is>
-          <t>HYDRAULIC HOSE 3/4 "</t>
+          <t>HYDRAULIC HOSE 1"</t>
         </is>
       </c>
     </row>
     <row r="3159">
       <c r="A3159" t="inlineStr">
         <is>
-          <t>471 TC- 16BX</t>
+          <t>471 TC- 20BX</t>
         </is>
       </c>
       <c r="B3159" t="inlineStr">
@@ -50498,14 +50498,14 @@
       </c>
       <c r="C3159" t="inlineStr">
         <is>
-          <t>HYDRAULIC HOSE 1"</t>
+          <t>HYDRAULIC HOSE 1 1/4"</t>
         </is>
       </c>
     </row>
     <row r="3160">
       <c r="A3160" t="inlineStr">
         <is>
-          <t>471 TC- 20BX</t>
+          <t>10643-4-4</t>
         </is>
       </c>
       <c r="B3160" t="inlineStr">
@@ -50515,14 +50515,14 @@
       </c>
       <c r="C3160" t="inlineStr">
         <is>
-          <t>HYDRAULIC HOSE 1 1/4"</t>
+          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1/4</t>
         </is>
       </c>
     </row>
     <row r="3161">
       <c r="A3161" t="inlineStr">
         <is>
-          <t>10643-4-4</t>
+          <t>10643-8-8</t>
         </is>
       </c>
       <c r="B3161" t="inlineStr">
@@ -50532,48 +50532,48 @@
       </c>
       <c r="C3161" t="inlineStr">
         <is>
-          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1/4</t>
+          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1/2</t>
         </is>
       </c>
     </row>
     <row r="3162">
       <c r="A3162" t="inlineStr">
         <is>
-          <t>10643-8-8</t>
+          <t>10643-12-12</t>
         </is>
       </c>
       <c r="B3162" t="inlineStr">
         <is>
-          <t>GENERAL</t>
+          <t>PARKER</t>
         </is>
       </c>
       <c r="C3162" t="inlineStr">
         <is>
-          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1/2</t>
+          <t>JIC 37`, FEMALE, SWIVEL, 90` ELBOW SIZE 3/4</t>
         </is>
       </c>
     </row>
     <row r="3163">
       <c r="A3163" t="inlineStr">
         <is>
-          <t>10643-12-12</t>
+          <t>10643-16-16</t>
         </is>
       </c>
       <c r="B3163" t="inlineStr">
         <is>
-          <t>PARKER</t>
+          <t>GENERAL</t>
         </is>
       </c>
       <c r="C3163" t="inlineStr">
         <is>
-          <t>JIC 37`, FEMALE, SWIVEL, 90` ELBOW SIZE 3/4</t>
+          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1"</t>
         </is>
       </c>
     </row>
     <row r="3164">
       <c r="A3164" t="inlineStr">
         <is>
-          <t>10643-16-16</t>
+          <t>10643-20-20</t>
         </is>
       </c>
       <c r="B3164" t="inlineStr">
@@ -50583,31 +50583,31 @@
       </c>
       <c r="C3164" t="inlineStr">
         <is>
-          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1"</t>
+          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1 1/4"</t>
         </is>
       </c>
     </row>
     <row r="3165">
       <c r="A3165" t="inlineStr">
         <is>
-          <t>10643-20-20</t>
+          <t>472 TC-20</t>
         </is>
       </c>
       <c r="B3165" t="inlineStr">
         <is>
-          <t>GENERAL</t>
+          <t>PARKER</t>
         </is>
       </c>
       <c r="C3165" t="inlineStr">
         <is>
-          <t>JIC 37`, FEMALE, SWIVEL, STRAIGHT SIZE 1 1/4"</t>
+          <t>HYDRAULIC HOSE 1 1/4 "</t>
         </is>
       </c>
     </row>
     <row r="3166">
       <c r="A3166" t="inlineStr">
         <is>
-          <t>472 TC-20</t>
+          <t>13943-8-8</t>
         </is>
       </c>
       <c r="B3166" t="inlineStr">
@@ -50617,14 +50617,14 @@
       </c>
       <c r="C3166" t="inlineStr">
         <is>
-          <t>HYDRAULIC HOSE 1 1/4 "</t>
+          <t>JIC 37`, FEMALE, SWIVEL, 90` ELBOW SIZE 1/2</t>
         </is>
       </c>
     </row>
     <row r="3167">
       <c r="A3167" t="inlineStr">
         <is>
-          <t>13943-8-8</t>
+          <t>13943-12-12</t>
         </is>
       </c>
       <c r="B3167" t="inlineStr">
@@ -50634,14 +50634,14 @@
       </c>
       <c r="C3167" t="inlineStr">
         <is>
-          <t>JIC 37`, FEMALE, SWIVEL, 90` ELBOW SIZE 1/2</t>
+          <t>JIC 37`, FEMALE, SWIVEL, 90` ELBOW SIZE 3/4</t>
         </is>
       </c>
     </row>
     <row r="3168">
       <c r="A3168" t="inlineStr">
         <is>
-          <t>13943-12-12</t>
+          <t>13943-16-16</t>
         </is>
       </c>
       <c r="B3168" t="inlineStr">
@@ -50650,23 +50650,6 @@
         </is>
       </c>
       <c r="C3168" t="inlineStr">
-        <is>
-          <t>JIC 37`, FEMALE, SWIVEL, 90` ELBOW SIZE 3/4</t>
-        </is>
-      </c>
-    </row>
-    <row r="3169">
-      <c r="A3169" t="inlineStr">
-        <is>
-          <t>13943-16-16</t>
-        </is>
-      </c>
-      <c r="B3169" t="inlineStr">
-        <is>
-          <t>PARKER</t>
-        </is>
-      </c>
-      <c r="C3169" t="inlineStr">
         <is>
           <t>JIC 37`, FEMALE, SWIVEL, 90` ELBOW SIZE 1 1/4"</t>
         </is>

</xml_diff>